<commit_message>
Adding the updated datasets excel
</commit_message>
<xml_diff>
--- a/data/datasets.xlsx
+++ b/data/datasets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kokul/Projects/GOMAP-enrich/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90B9C563-4FEC-264F-AA4F-C56A553031A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{268C94C9-4725-3E46-A47C-69EE8E0127C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{E467A60D-F69A-4F4A-9E6E-FC569BD129C9}"/>
+    <workbookView xWindow="15120" yWindow="760" windowWidth="15120" windowHeight="18880" xr2:uid="{E467A60D-F69A-4F4A-9E6E-FC569BD129C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="704" uniqueCount="278">
   <si>
     <t>Species</t>
   </si>
@@ -868,6 +868,9 @@
   </si>
   <si>
     <t>Wild_Tomato_SGN_LA716_June_2023_v2.r1.gaf.gz</t>
+  </si>
+  <si>
+    <t>CSS_ChrLev_20200506</t>
   </si>
 </sst>
 </file>
@@ -2305,6 +2308,12 @@
       <c r="C53" t="s">
         <v>269</v>
       </c>
+      <c r="D53" t="s">
+        <v>277</v>
+      </c>
+      <c r="E53" t="s">
+        <v>277</v>
+      </c>
       <c r="F53" t="s">
         <v>266</v>
       </c>

</xml_diff>